<commit_message>
vault backup: 2026-10-06 10:59:23
</commit_message>
<xml_diff>
--- a/01 Firma/Aquise Informationen.xlsx
+++ b/01 Firma/Aquise Informationen.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natgu\Documents\business-infos\01 Firma\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A80DB593-FB9D-42F6-B329-FE7F17A21AFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63D600E1-94D1-4EB6-AB24-DDD2E316E2FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-83" yWindow="0" windowWidth="10965" windowHeight="13763" xr2:uid="{3EA3A60B-FE93-4079-91CC-1389B61F5F98}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="53">
   <si>
     <t>Aquisen</t>
   </si>
@@ -675,7 +675,9 @@
       <c r="D3" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="2"/>
+      <c r="E3" s="2">
+        <v>46301</v>
+      </c>
       <c r="F3" t="s">
         <v>14</v>
       </c>
@@ -693,7 +695,12 @@
       <c r="D4" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="2"/>
+      <c r="E4" s="2">
+        <v>46301</v>
+      </c>
+      <c r="F4" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
@@ -708,7 +715,12 @@
       <c r="D5" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="2"/>
+      <c r="E5" s="2">
+        <v>46302</v>
+      </c>
+      <c r="F5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
@@ -723,7 +735,12 @@
       <c r="D6" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="2"/>
+      <c r="E6" s="2">
+        <v>46302</v>
+      </c>
+      <c r="F6" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
@@ -738,7 +755,12 @@
       <c r="D7" t="s">
         <v>4</v>
       </c>
-      <c r="E7" s="2"/>
+      <c r="E7" s="2">
+        <v>46302</v>
+      </c>
+      <c r="F7" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
@@ -753,7 +775,12 @@
       <c r="D8" t="s">
         <v>4</v>
       </c>
-      <c r="E8" s="2"/>
+      <c r="E8" s="2">
+        <v>46303</v>
+      </c>
+      <c r="F8" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
@@ -768,7 +795,12 @@
       <c r="D9" t="s">
         <v>4</v>
       </c>
-      <c r="E9" s="2"/>
+      <c r="E9" s="2">
+        <v>46305</v>
+      </c>
+      <c r="F9" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
@@ -783,7 +815,12 @@
       <c r="D10" t="s">
         <v>4</v>
       </c>
-      <c r="E10" s="2"/>
+      <c r="E10" s="2">
+        <v>46305</v>
+      </c>
+      <c r="F10" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
@@ -798,7 +835,12 @@
       <c r="D11" t="s">
         <v>4</v>
       </c>
-      <c r="E11" s="2"/>
+      <c r="E11" s="2">
+        <v>46305</v>
+      </c>
+      <c r="F11" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
@@ -813,7 +855,12 @@
       <c r="D12" t="s">
         <v>4</v>
       </c>
-      <c r="E12" s="2"/>
+      <c r="E12" s="2">
+        <v>46305</v>
+      </c>
+      <c r="F12" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
@@ -828,7 +875,12 @@
       <c r="D13" t="s">
         <v>4</v>
       </c>
-      <c r="E13" s="2"/>
+      <c r="E13" s="2">
+        <v>46305</v>
+      </c>
+      <c r="F13" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A14" t="s">

</xml_diff>

<commit_message>
vault backup: 2026-10-06 18:02:46
</commit_message>
<xml_diff>
--- a/01 Firma/Aquise Informationen.xlsx
+++ b/01 Firma/Aquise Informationen.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natgu\Documents\business-infos\01 Firma\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63D600E1-94D1-4EB6-AB24-DDD2E316E2FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50FB1B93-6478-44FF-A9CF-1A431635A368}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{3EA3A60B-FE93-4079-91CC-1389B61F5F98}"/>
   </bookViews>
@@ -204,7 +204,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -228,13 +228,26 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="24"/>
+      <color theme="0"/>
+      <name val="Arial Black"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF6600"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -250,11 +263,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -284,6 +303,13 @@
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFF6600"/>
+      <color rgb="FFFF9933"/>
+      <color rgb="FFFF9900"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -637,10 +663,15 @@
     <col min="5" max="5" width="13.73046875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A1" t="s">
+    <row r="1" spans="1:6" ht="36.4" x14ac:dyDescent="1.35">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
@@ -5068,6 +5099,9 @@
       <c r="E1380" s="2"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
   <dataValidations count="5">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D1381:D2011" xr:uid="{6C3AF1DC-FFEA-4827-8AF8-30DDDE6252EB}">
       <mc:AlternateContent xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">

</xml_diff>

<commit_message>
vault backup: 2026-10-07 08:47:29
</commit_message>
<xml_diff>
--- a/01 Firma/Aquise Informationen.xlsx
+++ b/01 Firma/Aquise Informationen.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natgu\Documents\business-infos\01 Firma\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50FB1B93-6478-44FF-A9CF-1A431635A368}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3938C6A2-9C4C-4D86-8BCB-0ADC75CDF8C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{3EA3A60B-FE93-4079-91CC-1389B61F5F98}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="53">
   <si>
     <t>Aquisen</t>
   </si>
@@ -926,7 +926,12 @@
       <c r="D14" t="s">
         <v>8</v>
       </c>
-      <c r="E14" s="2"/>
+      <c r="E14" s="2">
+        <v>46307</v>
+      </c>
+      <c r="F14" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A15" t="s">

</xml_diff>